<commit_message>
Do not charge Chris for January–April CIUDAD settlement.
Debt starts in May, the first month with Almacén Chris; regenerate the
rendition totals from May–July only.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Rendicion_CIUDAD_2026.xlsx
+++ b/CIUDAD/Rendicion_CIUDAD_2026.xlsx
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado 2026-09-10 · Fuente: Gastos_CIUDAD_1132_2026.xlsx · Servicios÷2 + Almacén÷2 − lo que cada uno ya pagó → quién le debe a quién</t>
+          <t>Generado 2026-09-11 · Fuente: Gastos_CIUDAD_1132_2026.xlsx · Servicios÷2 + Almacén÷2 − lo que cada uno ya pagó → quién le debe a quién</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Chris le debe a Sol $1.202.668</t>
+          <t>Sin cargo a Chris (aún no pasó almacén)</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Chris le debe a Sol $961.735</t>
+          <t>Sin cargo a Chris (aún no pasó almacén)</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Chris le debe a Sol $1.053.746</t>
+          <t>Sin cargo a Chris (aún no pasó almacén)</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Chris le debe a Sol $1.129.851</t>
+          <t>Sin cargo a Chris (aún no pasó almacén)</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       <c r="J17" s="11" t="n"/>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>Chris → Sol (meses completos): $7.328.677</t>
+          <t>Chris → Sol (desde 1er mes con almacén Chris): $2.980.677</t>
         </is>
       </c>
     </row>
@@ -1207,6 +1207,13 @@
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
+        <is>
+          <t>• 6) Enero–abril: NO se le cobra nada a Chris (todavía no había pasado gastos de almacén). La deuda arranca en mayo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>• Agosto–diciembre: almacén vacío / Telecentro proyectado — no liquidar hasta completar el mes.</t>
         </is>
@@ -4607,17 +4614,17 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-1202667</v>
+        <v>0</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>1202668</v>
+        <v>0</v>
       </c>
       <c r="D13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $1.202.668</t>
+          <t>→ Sin cargo a Chris (aún no pasó almacén)</t>
         </is>
       </c>
     </row>
@@ -6244,17 +6251,17 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-961735</v>
+        <v>0</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>961735</v>
+        <v>0</v>
       </c>
       <c r="D13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $961.735</t>
+          <t>→ Sin cargo a Chris (aún no pasó almacén)</t>
         </is>
       </c>
     </row>
@@ -7922,17 +7929,17 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-1053745</v>
+        <v>0</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>1053746</v>
+        <v>0</v>
       </c>
       <c r="D13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $1.053.746</t>
+          <t>→ Sin cargo a Chris (aún no pasó almacén)</t>
         </is>
       </c>
     </row>
@@ -9435,17 +9442,17 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-1129850</v>
+        <v>0</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>1129851</v>
+        <v>0</v>
       </c>
       <c r="D13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $1.129.851</t>
+          <t>→ Sin cargo a Chris (aún no pasó almacén)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate rendition after excluding Telecentro-only months.
January–April remain without Chris charges; debt totals May–July only.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Rendicion_CIUDAD_2026.xlsx
+++ b/CIUDAD/Rendicion_CIUDAD_2026.xlsx
@@ -2326,7 +2326,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $25.000</t>
+          <t>→ Mes incompleto — no liquidar aún</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2606,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $25.000</t>
+          <t>→ Mes incompleto — no liquidar aún</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $25.000</t>
+          <t>→ Mes incompleto — no liquidar aún</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3166,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $25.000</t>
+          <t>→ Mes incompleto — no liquidar aún</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>→ Chris le debe a Sol $25.000</t>
+          <t>→ Mes incompleto — no liquidar aún</t>
         </is>
       </c>
     </row>

</xml_diff>